<commit_message>
feat: enforce extraction allowlist and fix top-2 metric logic
Add EXTRACTION_SCENARIO_ALLOWLIST to prevent engineering-truth keys from reaching the LLM prompt, raising on unexpected scenario keys. Fix top-2 accuracy in CalculateMetrics to use containment check instead of set intersection, which is degenerate for n=3 alternatives. Refactor SensitivityAnalysis to use _build_config and add alpha sweep for value-function shape analysis.
</commit_message>
<xml_diff>
--- a/Output Files DeepSeek V4 Flash/sensitivity_analysis_deepseek.xlsx
+++ b/Output Files DeepSeek V4 Flash/sensitivity_analysis_deepseek.xlsx
@@ -413,914 +413,2459 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>scenario_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>weights_json</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>architecture</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>kendall_tau</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>spearman_rho</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>top1_accuracy</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>top2_accuracy</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>gap_rag_minus_pure</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>gap_param_minus_rag</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.159</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>0.1667</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.4</v>
       </c>
-      <c r="G2" t="n">
-        <v>1</v>
+      <c r="H2" t="n">
+        <v>0.7179</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.5469999999999999</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.3504</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>0.3692</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.5641</v>
       </c>
-      <c r="G3" t="n">
-        <v>1</v>
+      <c r="H3" t="n">
+        <v>0.8205</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.5469999999999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>baseline</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.8974</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>0.9103</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>0.9127999999999999</v>
       </c>
-      <c r="G4" t="n">
-        <v>1</v>
+      <c r="H4" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.5469999999999999</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>ene +0.05</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.35, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>0.2034</v>
       </c>
-      <c r="E5" t="n">
+      <c r="F5" t="n">
         <v>0.2231</v>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>0.4051</v>
       </c>
-      <c r="G5" t="n">
-        <v>1</v>
+      <c r="H5" t="n">
+        <v>0.7538</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0.1436</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.5333</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>ene +0.05</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.35, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>0.347</v>
       </c>
-      <c r="E6" t="n">
+      <c r="F6" t="n">
         <v>0.359</v>
       </c>
-      <c r="F6" t="n">
+      <c r="G6" t="n">
         <v>0.5538</v>
       </c>
-      <c r="G6" t="n">
-        <v>1</v>
+      <c r="H6" t="n">
+        <v>0.8256</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0.1436</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.5333</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>ene +0.05</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.35, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="E7" t="n">
         <v>0.8803</v>
       </c>
-      <c r="E7" t="n">
+      <c r="F7" t="n">
         <v>0.9</v>
       </c>
-      <c r="F7" t="n">
+      <c r="G7" t="n">
         <v>0.8974</v>
       </c>
-      <c r="G7" t="n">
-        <v>1</v>
+      <c r="H7" t="n">
+        <v>0.9795</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0.1436</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.5333</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>ene -0.05</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="E8" t="n">
+        <v>0.1316</v>
+      </c>
+      <c r="F8" t="n">
         <v>0.1385</v>
       </c>
-      <c r="E8" t="n">
-        <v>0.1462</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0.3795</v>
-      </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0.3744</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.6974</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0.2291</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.5709</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>ene -0.05</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>0.3675</v>
-      </c>
       <c r="E9" t="n">
-        <v>0.3923</v>
+        <v>0.3607</v>
       </c>
       <c r="F9" t="n">
-        <v>0.5641</v>
+        <v>0.3872</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0.5590000000000001</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.8615</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0.2291</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.5709</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>ene -0.05</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>0.9385</v>
-      </c>
       <c r="E10" t="n">
-        <v>0.9487</v>
+        <v>0.9316</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9487</v>
+        <v>0.9436</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0.9436</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.9949</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0.2291</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.5709</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>env +0.05</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.4, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="E11" t="n">
         <v>0.1761</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>0.1923</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>0.3846</v>
       </c>
-      <c r="G11" t="n">
-        <v>1</v>
+      <c r="H11" t="n">
+        <v>0.7282</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.5230999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>env +0.05</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.4, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="E12" t="n">
         <v>0.3675</v>
       </c>
-      <c r="E12" t="n">
+      <c r="F12" t="n">
         <v>0.3872</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>0.5692</v>
       </c>
-      <c r="G12" t="n">
-        <v>1</v>
+      <c r="H12" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.5230999999999999</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>env +0.05</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.4, "comfort": 0.183333, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="E13" t="n">
         <v>0.8905999999999999</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>0.9051</v>
       </c>
-      <c r="F13" t="n">
+      <c r="G13" t="n">
         <v>0.9077</v>
       </c>
-      <c r="G13" t="n">
-        <v>1</v>
+      <c r="H13" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.1914</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.5230999999999999</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>env -0.05</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.3, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>0.1385</v>
-      </c>
       <c r="E14" t="n">
-        <v>0.1436</v>
+        <v>0.135</v>
       </c>
       <c r="F14" t="n">
-        <v>0.3744</v>
+        <v>0.141</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0.3692</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.6974</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0.2052</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.5948</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>env -0.05</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.3, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>0.3436</v>
-      </c>
       <c r="E15" t="n">
-        <v>0.3692</v>
+        <v>0.3402</v>
       </c>
       <c r="F15" t="n">
-        <v>0.5436</v>
+        <v>0.3667</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>0.5385</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.8564000000000001</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0.2052</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.5948</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>env -0.05</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.3, "comfort": 0.216667, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>0.9385</v>
-      </c>
       <c r="E16" t="n">
-        <v>0.9513</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="F16" t="n">
         <v>0.9487</v>
       </c>
       <c r="G16" t="n">
+        <v>0.9436</v>
+      </c>
+      <c r="H16" t="n">
         <v>1</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0.2052</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.5948</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>com +0.05</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.25, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>0.1419</v>
-      </c>
       <c r="E17" t="n">
-        <v>0.1487</v>
+        <v>0.1385</v>
       </c>
       <c r="F17" t="n">
+        <v>0.1436</v>
+      </c>
+      <c r="G17" t="n">
         <v>0.3795</v>
       </c>
-      <c r="G17" t="n">
-        <v>1</v>
+      <c r="H17" t="n">
+        <v>0.7077</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.5778</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>com +0.05</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.25, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>0.3504</v>
-      </c>
       <c r="E18" t="n">
-        <v>0.3795</v>
+        <v>0.347</v>
       </c>
       <c r="F18" t="n">
+        <v>0.3769</v>
+      </c>
+      <c r="G18" t="n">
         <v>0.5590000000000001</v>
       </c>
-      <c r="G18" t="n">
-        <v>1</v>
+      <c r="H18" t="n">
+        <v>0.8512999999999999</v>
+      </c>
+      <c r="I18" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.5778</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>com +0.05</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.25, "practicality": 0.133333}</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D19" t="n">
+      <c r="E19" t="n">
+        <v>0.9248</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0.9359</v>
+      </c>
+      <c r="G19" t="n">
         <v>0.9282</v>
       </c>
-      <c r="E19" t="n">
-        <v>0.9409999999999999</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0.9282</v>
-      </c>
-      <c r="G19" t="n">
-        <v>1</v>
+      <c r="H19" t="n">
+        <v>0.9949</v>
+      </c>
+      <c r="I19" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.5778</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>com -0.05</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.15, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="E20" t="n">
         <v>0.2171</v>
       </c>
-      <c r="E20" t="n">
+      <c r="F20" t="n">
         <v>0.2359</v>
       </c>
-      <c r="F20" t="n">
+      <c r="G20" t="n">
         <v>0.4154</v>
       </c>
-      <c r="G20" t="n">
-        <v>1</v>
+      <c r="H20" t="n">
+        <v>0.7487</v>
+      </c>
+      <c r="I20" t="n">
+        <v>0.1402</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.5024999999999999</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>com -0.05</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.15, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="E21" t="n">
         <v>0.3573</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>0.3718</v>
       </c>
-      <c r="F21" t="n">
+      <c r="G21" t="n">
         <v>0.5692</v>
       </c>
-      <c r="G21" t="n">
-        <v>1</v>
+      <c r="H21" t="n">
+        <v>0.8256</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0.1402</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.5024999999999999</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>com -0.05</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.15, "practicality": 0.166667}</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D22" t="n">
+      <c r="E22" t="n">
         <v>0.8598</v>
       </c>
-      <c r="E22" t="n">
+      <c r="F22" t="n">
         <v>0.8794999999999999</v>
       </c>
-      <c r="F22" t="n">
+      <c r="G22" t="n">
         <v>0.8974</v>
       </c>
-      <c r="G22" t="n">
-        <v>1</v>
+      <c r="H22" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="I22" t="n">
+        <v>0.1402</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.5024999999999999</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>pra +0.05</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.2}</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="E23" t="n">
         <v>0.1214</v>
       </c>
-      <c r="E23" t="n">
+      <c r="F23" t="n">
         <v>0.1308</v>
       </c>
-      <c r="F23" t="n">
+      <c r="G23" t="n">
         <v>0.3436</v>
       </c>
-      <c r="G23" t="n">
-        <v>1</v>
+      <c r="H23" t="n">
+        <v>0.7026</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.5880000000000001</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>pra +0.05</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.2}</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D24" t="n">
+      <c r="E24" t="n">
         <v>0.3299</v>
       </c>
-      <c r="E24" t="n">
+      <c r="F24" t="n">
         <v>0.3487</v>
       </c>
-      <c r="F24" t="n">
+      <c r="G24" t="n">
         <v>0.5385</v>
       </c>
-      <c r="G24" t="n">
-        <v>1</v>
+      <c r="H24" t="n">
+        <v>0.8205</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.5880000000000001</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>pra +0.05</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.283333, "environmental": 0.333333, "comfort": 0.183333, "practicality": 0.2}</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D25" t="n">
+      <c r="E25" t="n">
         <v>0.9179</v>
       </c>
-      <c r="E25" t="n">
+      <c r="F25" t="n">
         <v>0.9308</v>
       </c>
-      <c r="F25" t="n">
+      <c r="G25" t="n">
         <v>0.9282</v>
       </c>
-      <c r="G25" t="n">
-        <v>1</v>
+      <c r="H25" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.2085</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.5880000000000001</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>pra -0.05</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.1}</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="E26" t="n">
         <v>0.1966</v>
       </c>
-      <c r="E26" t="n">
+      <c r="F26" t="n">
         <v>0.2154</v>
       </c>
-      <c r="F26" t="n">
+      <c r="G26" t="n">
         <v>0.4103</v>
       </c>
-      <c r="G26" t="n">
-        <v>1</v>
+      <c r="H26" t="n">
+        <v>0.7436</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.1675</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.5299</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>pra -0.05</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.1}</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="E27" t="n">
         <v>0.3641</v>
       </c>
-      <c r="E27" t="n">
+      <c r="F27" t="n">
         <v>0.3821</v>
       </c>
-      <c r="F27" t="n">
+      <c r="G27" t="n">
         <v>0.5641</v>
       </c>
-      <c r="G27" t="n">
-        <v>1</v>
+      <c r="H27" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.1675</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.5299</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>pra -0.05</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.316667, "environmental": 0.366667, "comfort": 0.216667, "practicality": 0.1}</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D28" t="n">
+      <c r="E28" t="n">
         <v>0.894</v>
       </c>
-      <c r="E28" t="n">
+      <c r="F28" t="n">
         <v>0.9077</v>
       </c>
-      <c r="F28" t="n">
+      <c r="G28" t="n">
         <v>0.9179</v>
       </c>
-      <c r="G28" t="n">
-        <v>1</v>
+      <c r="H28" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.1675</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.5299</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>equal</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.25, "comfort": 0.25, "practicality": 0.25}</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Direct_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D29" t="n">
+      <c r="E29" t="n">
         <v>0.1214</v>
       </c>
-      <c r="E29" t="n">
+      <c r="F29" t="n">
         <v>0.1256</v>
       </c>
-      <c r="F29" t="n">
+      <c r="G29" t="n">
         <v>0.3795</v>
       </c>
-      <c r="G29" t="n">
-        <v>1</v>
+      <c r="H29" t="n">
+        <v>0.6923</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0.2154</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.5846</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>equal</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.25, "comfort": 0.25, "practicality": 0.25}</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Example-Guided_LLM_Scoring</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="E30" t="n">
         <v>0.3368</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>0.3564</v>
       </c>
-      <c r="F30" t="n">
+      <c r="G30" t="n">
         <v>0.5077</v>
       </c>
-      <c r="G30" t="n">
-        <v>1</v>
+      <c r="H30" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0.2154</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.5846</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>equal</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>{"energy_cost": 0.25, "environmental": 0.25, "comfort": 0.25, "practicality": 0.25}</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>LLM-Parameterized_Reference_Scoring</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="E31" t="n">
         <v>0.9214</v>
       </c>
-      <c r="E31" t="n">
+      <c r="F31" t="n">
         <v>0.9359</v>
       </c>
-      <c r="F31" t="n">
+      <c r="G31" t="n">
         <v>0.9538</v>
       </c>
-      <c r="G31" t="n">
+      <c r="H31" t="n">
+        <v>0.9949</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0.2154</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.5846</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>merec pooled</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>0.3265</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0.3564</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0.5026</v>
+      </c>
+      <c r="H32" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0.4718</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>merec pooled</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>0.4838</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.5282</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0.6205000000000001</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0.8974</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0.4718</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>merec pooled</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>0.9556</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0.9667</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0.9385</v>
+      </c>
+      <c r="H34" t="n">
         <v>1</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0.1573</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0.4718</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>merec hvac-vec</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>0.5282</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0.5692</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0.6768999999999999</v>
+      </c>
+      <c r="H35" t="n">
+        <v>0.8872</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-0.05809999999999998</v>
+      </c>
+      <c r="J35" t="n">
+        <v>0.4990999999999999</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>merec hvac-vec</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.4701</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0.5154</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.5795</v>
+      </c>
+      <c r="H36" t="n">
+        <v>0.9026</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-0.05809999999999998</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.4990999999999999</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>merec hvac-vec</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.9769</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.959</v>
+      </c>
+      <c r="H37" t="n">
+        <v>1</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-0.05809999999999998</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.4990999999999999</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>merec appliance-vec</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.2171</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0.2256</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.4359</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0.7282</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.2838000000000001</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.4136</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>merec appliance-vec</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.5009</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0.5231</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.6513</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0.8769</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.2838000000000001</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.4136</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>merec appliance-vec</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.9145</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0.9333</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.9077</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.2838000000000001</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.4136</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>merec shower-vec</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.1043</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.1154</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.3436</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0.6974</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.1948</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.6086</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>merec shower-vec</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.2991</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0.3231</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.4872</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0.8308</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.1948</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.6086</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>merec shower-vec</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.9077</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0.9256</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.9282</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0.9949</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.1948</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.6086</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>merec per-type</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.4564</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0.4872</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.6051</v>
+      </c>
+      <c r="H44" t="n">
+        <v>0.8462</v>
+      </c>
+      <c r="I44" t="n">
+        <v>-0.03759999999999997</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.5197000000000001</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>merec per-type</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.4188</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.4513</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.5282</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.8974</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-0.03759999999999997</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.5197000000000001</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>merec per-type</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>0.9385</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0.9487</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0.9538</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0.9949</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-0.03759999999999997</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0.5197000000000001</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>entropy pooled</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0.1487</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0.1564</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0.3795</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0.7128</v>
+      </c>
+      <c r="I47" t="n">
+        <v>0.1846</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.5402</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>entropy pooled</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>0.3333</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0.3538</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0.5436</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0.8256</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.1846</v>
+      </c>
+      <c r="J48" t="n">
+        <v>0.5402</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>entropy pooled</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0.8897</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0.9026</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.1846</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0.5402</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>entropy hvac-vec</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>0.2137</v>
+      </c>
+      <c r="F50" t="n">
+        <v>0.2231</v>
+      </c>
+      <c r="G50" t="n">
+        <v>0.4513</v>
+      </c>
+      <c r="H50" t="n">
+        <v>0.7487</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.1607</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.4991</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>entropy hvac-vec</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>0.3744</v>
+      </c>
+      <c r="F51" t="n">
+        <v>0.3974</v>
+      </c>
+      <c r="G51" t="n">
+        <v>0.5846</v>
+      </c>
+      <c r="H51" t="n">
+        <v>0.8512999999999999</v>
+      </c>
+      <c r="I51" t="n">
+        <v>0.1607</v>
+      </c>
+      <c r="J51" t="n">
+        <v>0.4991</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>entropy hvac-vec</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>0.8735000000000001</v>
+      </c>
+      <c r="F52" t="n">
+        <v>0.8974</v>
+      </c>
+      <c r="G52" t="n">
+        <v>0.8769</v>
+      </c>
+      <c r="H52" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="I52" t="n">
+        <v>0.1607</v>
+      </c>
+      <c r="J52" t="n">
+        <v>0.4991</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>entropy appliance-vec</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>0.1385</v>
+      </c>
+      <c r="F53" t="n">
+        <v>0.1487</v>
+      </c>
+      <c r="G53" t="n">
+        <v>0.3949</v>
+      </c>
+      <c r="H53" t="n">
+        <v>0.6872</v>
+      </c>
+      <c r="I53" t="n">
+        <v>0.2359</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0.4923</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>entropy appliance-vec</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>0.3744</v>
+      </c>
+      <c r="F54" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="G54" t="n">
+        <v>0.5897</v>
+      </c>
+      <c r="H54" t="n">
+        <v>0.8205</v>
+      </c>
+      <c r="I54" t="n">
+        <v>0.2359</v>
+      </c>
+      <c r="J54" t="n">
+        <v>0.4923</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>entropy appliance-vec</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="F55" t="n">
+        <v>0.8821</v>
+      </c>
+      <c r="G55" t="n">
+        <v>0.8974</v>
+      </c>
+      <c r="H55" t="n">
+        <v>0.9692</v>
+      </c>
+      <c r="I55" t="n">
+        <v>0.2359</v>
+      </c>
+      <c r="J55" t="n">
+        <v>0.4923</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>entropy shower-vec</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>0.1761</v>
+      </c>
+      <c r="F56" t="n">
+        <v>0.1872</v>
+      </c>
+      <c r="G56" t="n">
+        <v>0.3795</v>
+      </c>
+      <c r="H56" t="n">
+        <v>0.7077</v>
+      </c>
+      <c r="I56" t="n">
+        <v>0.1538</v>
+      </c>
+      <c r="J56" t="n">
+        <v>0.5367999999999999</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>entropy shower-vec</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>0.3299</v>
+      </c>
+      <c r="F57" t="n">
+        <v>0.3462</v>
+      </c>
+      <c r="G57" t="n">
+        <v>0.5487</v>
+      </c>
+      <c r="H57" t="n">
+        <v>0.8154</v>
+      </c>
+      <c r="I57" t="n">
+        <v>0.1538</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.5367999999999999</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>entropy shower-vec</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="F58" t="n">
+        <v>0.8846000000000001</v>
+      </c>
+      <c r="G58" t="n">
+        <v>0.8923</v>
+      </c>
+      <c r="H58" t="n">
+        <v>0.9744</v>
+      </c>
+      <c r="I58" t="n">
+        <v>0.1538</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0.5367999999999999</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>entropy per-type</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>0.0974</v>
+      </c>
+      <c r="F59" t="n">
+        <v>0.1026</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0.3795</v>
+      </c>
+      <c r="H59" t="n">
+        <v>0.6974</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.2975</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0.5094000000000001</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>entropy per-type</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>0.3949</v>
+      </c>
+      <c r="F60" t="n">
+        <v>0.4205</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0.5949</v>
+      </c>
+      <c r="H60" t="n">
+        <v>0.8667</v>
+      </c>
+      <c r="I60" t="n">
+        <v>0.2975</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0.5094000000000001</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>entropy per-type</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>0.9043</v>
+      </c>
+      <c r="F61" t="n">
+        <v>0.9205</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0.9282</v>
+      </c>
+      <c r="H61" t="n">
+        <v>0.9897</v>
+      </c>
+      <c r="I61" t="n">
+        <v>0.2975</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0.5094000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
reran everything & paper audit.
</commit_message>
<xml_diff>
--- a/Output Files DeepSeek V4 Flash/sensitivity_analysis_deepseek.xlsx
+++ b/Output Files DeepSeek V4 Flash/sensitivity_analysis_deepseek.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -490,22 +490,22 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>0.159</v>
+        <v>0.144</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1667</v>
+        <v>0.14522</v>
       </c>
       <c r="G2" t="n">
-        <v>0.4</v>
+        <v>0.36682</v>
       </c>
       <c r="H2" t="n">
-        <v>0.7179</v>
+        <v>0.7221</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1914</v>
+        <v>0.18386</v>
       </c>
       <c r="J2" t="n">
-        <v>0.5469999999999999</v>
+        <v>0.56948</v>
       </c>
     </row>
     <row r="3">
@@ -530,22 +530,22 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>0.3504</v>
+        <v>0.32786</v>
       </c>
       <c r="F3" t="n">
-        <v>0.3692</v>
+        <v>0.35384</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5641</v>
+        <v>0.5446</v>
       </c>
       <c r="H3" t="n">
-        <v>0.8205</v>
+        <v>0.8154</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1914</v>
+        <v>0.18386</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5469999999999999</v>
+        <v>0.56948</v>
       </c>
     </row>
     <row r="4">
@@ -570,22 +570,22 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>0.8974</v>
+        <v>0.89734</v>
       </c>
       <c r="F4" t="n">
-        <v>0.9103</v>
+        <v>0.9101399999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>0.9127999999999999</v>
+        <v>0.90762</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9744</v>
+        <v>0.9774200000000001</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1914</v>
+        <v>0.18386</v>
       </c>
       <c r="J4" t="n">
-        <v>0.5469999999999999</v>
+        <v>0.56948</v>
       </c>
     </row>
     <row r="5">
@@ -610,22 +610,22 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>0.2034</v>
+        <v>0.20258</v>
       </c>
       <c r="F5" t="n">
-        <v>0.2231</v>
+        <v>0.20982</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4051</v>
+        <v>0.4091799999999999</v>
       </c>
       <c r="H5" t="n">
-        <v>0.7538</v>
+        <v>0.7531199999999999</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1436</v>
+        <v>0.13346</v>
       </c>
       <c r="J5" t="n">
-        <v>0.5333</v>
+        <v>0.54144</v>
       </c>
     </row>
     <row r="6">
@@ -650,22 +650,22 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>0.347</v>
+        <v>0.33604</v>
       </c>
       <c r="F6" t="n">
-        <v>0.359</v>
+        <v>0.35692</v>
       </c>
       <c r="G6" t="n">
-        <v>0.5538</v>
+        <v>0.5497400000000001</v>
       </c>
       <c r="H6" t="n">
-        <v>0.8256</v>
+        <v>0.8194800000000001</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1436</v>
+        <v>0.13346</v>
       </c>
       <c r="J6" t="n">
-        <v>0.5333</v>
+        <v>0.54144</v>
       </c>
     </row>
     <row r="7">
@@ -690,22 +690,22 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>0.8803</v>
+        <v>0.87748</v>
       </c>
       <c r="F7" t="n">
-        <v>0.9</v>
+        <v>0.8947799999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>0.8974</v>
+        <v>0.8942399999999999</v>
       </c>
       <c r="H7" t="n">
-        <v>0.9795</v>
+        <v>0.9784600000000001</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1436</v>
+        <v>0.13346</v>
       </c>
       <c r="J7" t="n">
-        <v>0.5333</v>
+        <v>0.54144</v>
       </c>
     </row>
     <row r="8">
@@ -730,22 +730,22 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.1316</v>
+        <v>0.12056</v>
       </c>
       <c r="F8" t="n">
-        <v>0.1385</v>
+        <v>0.12146</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3744</v>
+        <v>0.3565</v>
       </c>
       <c r="H8" t="n">
-        <v>0.6974</v>
+        <v>0.71696</v>
       </c>
       <c r="I8" t="n">
-        <v>0.2291</v>
+        <v>0.21824</v>
       </c>
       <c r="J8" t="n">
-        <v>0.5709</v>
+        <v>0.5763</v>
       </c>
     </row>
     <row r="9">
@@ -770,22 +770,22 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>0.3607</v>
+        <v>0.3388</v>
       </c>
       <c r="F9" t="n">
-        <v>0.3872</v>
+        <v>0.36922</v>
       </c>
       <c r="G9" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.5374399999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>0.8615</v>
+        <v>0.8389800000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>0.2291</v>
+        <v>0.21824</v>
       </c>
       <c r="J9" t="n">
-        <v>0.5709</v>
+        <v>0.5763</v>
       </c>
     </row>
     <row r="10">
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>0.9316</v>
+        <v>0.9151</v>
       </c>
       <c r="F10" t="n">
-        <v>0.9436</v>
+        <v>0.9281200000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>0.9436</v>
+        <v>0.9301600000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>0.9949</v>
+        <v>0.9907599999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2291</v>
+        <v>0.21824</v>
       </c>
       <c r="J10" t="n">
-        <v>0.5709</v>
+        <v>0.5763</v>
       </c>
     </row>
     <row r="11">
@@ -850,22 +850,22 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>0.1761</v>
+        <v>0.17502</v>
       </c>
       <c r="F11" t="n">
-        <v>0.1923</v>
+        <v>0.17832</v>
       </c>
       <c r="G11" t="n">
-        <v>0.3846</v>
+        <v>0.3813</v>
       </c>
       <c r="H11" t="n">
-        <v>0.7282</v>
+        <v>0.73454</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1914</v>
+        <v>0.16788</v>
       </c>
       <c r="J11" t="n">
-        <v>0.5230999999999999</v>
+        <v>0.54416</v>
       </c>
     </row>
     <row r="12">
@@ -890,22 +890,22 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>0.3675</v>
+        <v>0.3429</v>
       </c>
       <c r="F12" t="n">
-        <v>0.3872</v>
+        <v>0.3672000000000001</v>
       </c>
       <c r="G12" t="n">
-        <v>0.5692</v>
+        <v>0.5599999999999999</v>
       </c>
       <c r="H12" t="n">
-        <v>0.8308</v>
+        <v>0.8215199999999999</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1914</v>
+        <v>0.16788</v>
       </c>
       <c r="J12" t="n">
-        <v>0.5230999999999999</v>
+        <v>0.54416</v>
       </c>
     </row>
     <row r="13">
@@ -930,22 +930,22 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>0.8905999999999999</v>
+        <v>0.88706</v>
       </c>
       <c r="F13" t="n">
-        <v>0.9051</v>
+        <v>0.90452</v>
       </c>
       <c r="G13" t="n">
-        <v>0.9077</v>
+        <v>0.8942600000000001</v>
       </c>
       <c r="H13" t="n">
-        <v>0.9744</v>
+        <v>0.9784600000000001</v>
       </c>
       <c r="I13" t="n">
-        <v>0.1914</v>
+        <v>0.16788</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5230999999999999</v>
+        <v>0.54416</v>
       </c>
     </row>
     <row r="14">
@@ -970,22 +970,22 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>0.135</v>
+        <v>0.12476</v>
       </c>
       <c r="F14" t="n">
-        <v>0.141</v>
+        <v>0.1277</v>
       </c>
       <c r="G14" t="n">
-        <v>0.3692</v>
+        <v>0.3565</v>
       </c>
       <c r="H14" t="n">
-        <v>0.6974</v>
+        <v>0.71594</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2052</v>
+        <v>0.19694</v>
       </c>
       <c r="J14" t="n">
-        <v>0.5948</v>
+        <v>0.5947999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -1010,22 +1010,22 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>0.3402</v>
+        <v>0.3217</v>
       </c>
       <c r="F15" t="n">
-        <v>0.3667</v>
+        <v>0.3518</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5385</v>
+        <v>0.52718</v>
       </c>
       <c r="H15" t="n">
-        <v>0.8564000000000001</v>
+        <v>0.8369399999999999</v>
       </c>
       <c r="I15" t="n">
-        <v>0.2052</v>
+        <v>0.19694</v>
       </c>
       <c r="J15" t="n">
-        <v>0.5948</v>
+        <v>0.5947999999999999</v>
       </c>
     </row>
     <row r="16">
@@ -1050,22 +1050,22 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>0.9350000000000001</v>
+        <v>0.9164999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9487</v>
+        <v>0.92864</v>
       </c>
       <c r="G16" t="n">
-        <v>0.9436</v>
+        <v>0.93122</v>
       </c>
       <c r="H16" t="n">
-        <v>1</v>
+        <v>0.9907599999999999</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2052</v>
+        <v>0.19694</v>
       </c>
       <c r="J16" t="n">
-        <v>0.5948</v>
+        <v>0.5947999999999999</v>
       </c>
     </row>
     <row r="17">
@@ -1090,22 +1090,22 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>0.1385</v>
+        <v>0.1144</v>
       </c>
       <c r="F17" t="n">
-        <v>0.1436</v>
+        <v>0.11582</v>
       </c>
       <c r="G17" t="n">
-        <v>0.3795</v>
+        <v>0.35546</v>
       </c>
       <c r="H17" t="n">
-        <v>0.7077</v>
+        <v>0.7149799999999999</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2085</v>
+        <v>0.20662</v>
       </c>
       <c r="J17" t="n">
-        <v>0.5778</v>
+        <v>0.5879400000000001</v>
       </c>
     </row>
     <row r="18">
@@ -1130,22 +1130,22 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.347</v>
+        <v>0.32102</v>
       </c>
       <c r="F18" t="n">
-        <v>0.3769</v>
+        <v>0.35538</v>
       </c>
       <c r="G18" t="n">
-        <v>0.5590000000000001</v>
+        <v>0.5312800000000001</v>
       </c>
       <c r="H18" t="n">
-        <v>0.8512999999999999</v>
+        <v>0.8338599999999999</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2085</v>
+        <v>0.20662</v>
       </c>
       <c r="J18" t="n">
-        <v>0.5778</v>
+        <v>0.5879400000000001</v>
       </c>
     </row>
     <row r="19">
@@ -1170,22 +1170,22 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>0.9248</v>
+        <v>0.9089600000000001</v>
       </c>
       <c r="F19" t="n">
-        <v>0.9359</v>
+        <v>0.9214399999999999</v>
       </c>
       <c r="G19" t="n">
-        <v>0.9282</v>
+        <v>0.9209400000000001</v>
       </c>
       <c r="H19" t="n">
-        <v>0.9949</v>
+        <v>0.9866200000000001</v>
       </c>
       <c r="I19" t="n">
-        <v>0.2085</v>
+        <v>0.20662</v>
       </c>
       <c r="J19" t="n">
-        <v>0.5778</v>
+        <v>0.5879400000000001</v>
       </c>
     </row>
     <row r="20">
@@ -1210,22 +1210,22 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.2171</v>
+        <v>0.19906</v>
       </c>
       <c r="F20" t="n">
-        <v>0.2359</v>
+        <v>0.20664</v>
       </c>
       <c r="G20" t="n">
-        <v>0.4154</v>
+        <v>0.39672</v>
       </c>
       <c r="H20" t="n">
-        <v>0.7487</v>
+        <v>0.7448599999999999</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1402</v>
+        <v>0.14248</v>
       </c>
       <c r="J20" t="n">
-        <v>0.5024999999999999</v>
+        <v>0.5235999999999998</v>
       </c>
     </row>
     <row r="21">
@@ -1250,22 +1250,22 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.3573</v>
+        <v>0.34154</v>
       </c>
       <c r="F21" t="n">
-        <v>0.3718</v>
+        <v>0.3595</v>
       </c>
       <c r="G21" t="n">
-        <v>0.5692</v>
+        <v>0.55794</v>
       </c>
       <c r="H21" t="n">
-        <v>0.8256</v>
+        <v>0.82256</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1402</v>
+        <v>0.14248</v>
       </c>
       <c r="J21" t="n">
-        <v>0.5024999999999999</v>
+        <v>0.5235999999999998</v>
       </c>
     </row>
     <row r="22">
@@ -1290,22 +1290,22 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>0.8598</v>
+        <v>0.8651399999999999</v>
       </c>
       <c r="F22" t="n">
-        <v>0.8794999999999999</v>
+        <v>0.88192</v>
       </c>
       <c r="G22" t="n">
-        <v>0.8974</v>
+        <v>0.8963000000000001</v>
       </c>
       <c r="H22" t="n">
-        <v>0.9692</v>
+        <v>0.9712400000000001</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1402</v>
+        <v>0.14248</v>
       </c>
       <c r="J22" t="n">
-        <v>0.5024999999999999</v>
+        <v>0.5235999999999998</v>
       </c>
     </row>
     <row r="23">
@@ -1330,22 +1330,22 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>0.1214</v>
+        <v>0.11786</v>
       </c>
       <c r="F23" t="n">
-        <v>0.1308</v>
+        <v>0.12046</v>
       </c>
       <c r="G23" t="n">
-        <v>0.3436</v>
+        <v>0.34826</v>
       </c>
       <c r="H23" t="n">
-        <v>0.7026</v>
+        <v>0.7179800000000001</v>
       </c>
       <c r="I23" t="n">
-        <v>0.2085</v>
+        <v>0.1929</v>
       </c>
       <c r="J23" t="n">
-        <v>0.5880000000000001</v>
+        <v>0.59272</v>
       </c>
     </row>
     <row r="24">
@@ -1370,22 +1370,22 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.3299</v>
+        <v>0.31076</v>
       </c>
       <c r="F24" t="n">
-        <v>0.3487</v>
+        <v>0.33384</v>
       </c>
       <c r="G24" t="n">
-        <v>0.5385</v>
+        <v>0.5210399999999999</v>
       </c>
       <c r="H24" t="n">
-        <v>0.8205</v>
+        <v>0.8164200000000001</v>
       </c>
       <c r="I24" t="n">
-        <v>0.2085</v>
+        <v>0.1929</v>
       </c>
       <c r="J24" t="n">
-        <v>0.5880000000000001</v>
+        <v>0.59272</v>
       </c>
     </row>
     <row r="25">
@@ -1410,22 +1410,22 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>0.9179</v>
+        <v>0.9034800000000001</v>
       </c>
       <c r="F25" t="n">
-        <v>0.9308</v>
+        <v>0.9193999999999999</v>
       </c>
       <c r="G25" t="n">
-        <v>0.9282</v>
+        <v>0.9168200000000001</v>
       </c>
       <c r="H25" t="n">
-        <v>0.9897</v>
+        <v>0.99178</v>
       </c>
       <c r="I25" t="n">
-        <v>0.2085</v>
+        <v>0.1929</v>
       </c>
       <c r="J25" t="n">
-        <v>0.5880000000000001</v>
+        <v>0.59272</v>
       </c>
     </row>
     <row r="26">
@@ -1450,22 +1450,22 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>0.1966</v>
+        <v>0.1833</v>
       </c>
       <c r="F26" t="n">
-        <v>0.2154</v>
+        <v>0.18866</v>
       </c>
       <c r="G26" t="n">
-        <v>0.4103</v>
+        <v>0.39266</v>
       </c>
       <c r="H26" t="n">
-        <v>0.7436</v>
+        <v>0.74282</v>
       </c>
       <c r="I26" t="n">
-        <v>0.1675</v>
+        <v>0.16164</v>
       </c>
       <c r="J26" t="n">
-        <v>0.5299</v>
+        <v>0.5537400000000001</v>
       </c>
     </row>
     <row r="27">
@@ -1490,22 +1490,22 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>0.3641</v>
+        <v>0.34494</v>
       </c>
       <c r="F27" t="n">
-        <v>0.3821</v>
+        <v>0.36668</v>
       </c>
       <c r="G27" t="n">
-        <v>0.5641</v>
+        <v>0.55076</v>
       </c>
       <c r="H27" t="n">
-        <v>0.8308</v>
+        <v>0.8215600000000001</v>
       </c>
       <c r="I27" t="n">
-        <v>0.1675</v>
+        <v>0.16164</v>
       </c>
       <c r="J27" t="n">
-        <v>0.5299</v>
+        <v>0.5537400000000001</v>
       </c>
     </row>
     <row r="28">
@@ -1530,22 +1530,22 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>0.894</v>
+        <v>0.89868</v>
       </c>
       <c r="F28" t="n">
-        <v>0.9077</v>
+        <v>0.91478</v>
       </c>
       <c r="G28" t="n">
-        <v>0.9179</v>
+        <v>0.90862</v>
       </c>
       <c r="H28" t="n">
-        <v>0.9744</v>
+        <v>0.98256</v>
       </c>
       <c r="I28" t="n">
-        <v>0.1675</v>
+        <v>0.16164</v>
       </c>
       <c r="J28" t="n">
-        <v>0.5299</v>
+        <v>0.5537400000000001</v>
       </c>
     </row>
     <row r="29">
@@ -1570,22 +1570,22 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>0.1214</v>
+        <v>0.11302</v>
       </c>
       <c r="F29" t="n">
-        <v>0.1256</v>
+        <v>0.11686</v>
       </c>
       <c r="G29" t="n">
-        <v>0.3795</v>
+        <v>0.3679</v>
       </c>
       <c r="H29" t="n">
-        <v>0.6923</v>
+        <v>0.7231799999999999</v>
       </c>
       <c r="I29" t="n">
-        <v>0.2154</v>
+        <v>0.20322</v>
       </c>
       <c r="J29" t="n">
-        <v>0.5846</v>
+        <v>0.5975</v>
       </c>
     </row>
     <row r="30">
@@ -1610,22 +1610,22 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>0.3368</v>
+        <v>0.31624</v>
       </c>
       <c r="F30" t="n">
-        <v>0.3564</v>
+        <v>0.3446</v>
       </c>
       <c r="G30" t="n">
-        <v>0.5077</v>
+        <v>0.5220399999999999</v>
       </c>
       <c r="H30" t="n">
-        <v>0.841</v>
+        <v>0.82872</v>
       </c>
       <c r="I30" t="n">
-        <v>0.2154</v>
+        <v>0.20322</v>
       </c>
       <c r="J30" t="n">
-        <v>0.5846</v>
+        <v>0.5975</v>
       </c>
     </row>
     <row r="31">
@@ -1650,22 +1650,22 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.9214</v>
+        <v>0.91374</v>
       </c>
       <c r="F31" t="n">
-        <v>0.9359</v>
+        <v>0.9301600000000001</v>
       </c>
       <c r="G31" t="n">
-        <v>0.9538</v>
+        <v>0.9373400000000001</v>
       </c>
       <c r="H31" t="n">
-        <v>0.9949</v>
+        <v>0.99382</v>
       </c>
       <c r="I31" t="n">
-        <v>0.2154</v>
+        <v>0.20322</v>
       </c>
       <c r="J31" t="n">
-        <v>0.5846</v>
+        <v>0.5975</v>
       </c>
     </row>
     <row r="32">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+          <t>{"energy_cost": 0.194172, "environmental": 0.131673, "comfort": 0.401912, "practicality": 0.272243}</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1690,22 +1690,22 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>0.3265</v>
+        <v>0.21884</v>
       </c>
       <c r="F32" t="n">
-        <v>0.3564</v>
+        <v>0.24516</v>
       </c>
       <c r="G32" t="n">
-        <v>0.5026</v>
+        <v>0.4347800000000001</v>
       </c>
       <c r="H32" t="n">
-        <v>0.8</v>
+        <v>0.7757400000000001</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1573</v>
+        <v>0.20954</v>
       </c>
       <c r="J32" t="n">
-        <v>0.4718</v>
+        <v>0.51616</v>
       </c>
     </row>
     <row r="33">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+          <t>{"energy_cost": 0.194172, "environmental": 0.131673, "comfort": 0.401912, "practicality": 0.272243}</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1730,22 +1730,22 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>0.4838</v>
+        <v>0.42838</v>
       </c>
       <c r="F33" t="n">
-        <v>0.5282</v>
+        <v>0.46258</v>
       </c>
       <c r="G33" t="n">
-        <v>0.6205000000000001</v>
+        <v>0.5825600000000001</v>
       </c>
       <c r="H33" t="n">
-        <v>0.8974</v>
+        <v>0.8656200000000001</v>
       </c>
       <c r="I33" t="n">
-        <v>0.1573</v>
+        <v>0.20954</v>
       </c>
       <c r="J33" t="n">
-        <v>0.4718</v>
+        <v>0.51616</v>
       </c>
     </row>
     <row r="34">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.19356, "environmental": 0.131075, "comfort": 0.40357, "practicality": 0.271796}</t>
+          <t>{"energy_cost": 0.194172, "environmental": 0.131673, "comfort": 0.401912, "practicality": 0.272243}</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1770,22 +1770,22 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>0.9556</v>
+        <v>0.9445399999999999</v>
       </c>
       <c r="F34" t="n">
-        <v>0.9667</v>
+        <v>0.9583999999999999</v>
       </c>
       <c r="G34" t="n">
-        <v>0.9385</v>
+        <v>0.93018</v>
       </c>
       <c r="H34" t="n">
         <v>1</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1573</v>
+        <v>0.20954</v>
       </c>
       <c r="J34" t="n">
-        <v>0.4718</v>
+        <v>0.51616</v>
       </c>
     </row>
     <row r="35">
@@ -1810,22 +1810,22 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>0.5282</v>
+        <v>0.3331</v>
       </c>
       <c r="F35" t="n">
-        <v>0.5692</v>
+        <v>0.36132</v>
       </c>
       <c r="G35" t="n">
-        <v>0.6768999999999999</v>
+        <v>0.5359999999999999</v>
       </c>
       <c r="H35" t="n">
-        <v>0.8872</v>
+        <v>0.8273999999999999</v>
       </c>
       <c r="I35" t="n">
-        <v>-0.05809999999999998</v>
+        <v>0.10688</v>
       </c>
       <c r="J35" t="n">
-        <v>0.4990999999999999</v>
+        <v>0.5312599999999998</v>
       </c>
     </row>
     <row r="36">
@@ -1850,22 +1850,22 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>0.4701</v>
+        <v>0.43998</v>
       </c>
       <c r="F36" t="n">
-        <v>0.5154</v>
+        <v>0.4749</v>
       </c>
       <c r="G36" t="n">
-        <v>0.5795</v>
+        <v>0.5815399999999999</v>
       </c>
       <c r="H36" t="n">
-        <v>0.9026</v>
+        <v>0.8738400000000001</v>
       </c>
       <c r="I36" t="n">
-        <v>-0.05809999999999998</v>
+        <v>0.10688</v>
       </c>
       <c r="J36" t="n">
-        <v>0.4990999999999999</v>
+        <v>0.5312599999999998</v>
       </c>
     </row>
     <row r="37">
@@ -1890,22 +1890,22 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.9692</v>
+        <v>0.9712399999999999</v>
       </c>
       <c r="F37" t="n">
-        <v>0.9769</v>
+        <v>0.97844</v>
       </c>
       <c r="G37" t="n">
-        <v>0.959</v>
+        <v>0.961</v>
       </c>
       <c r="H37" t="n">
         <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>-0.05809999999999998</v>
+        <v>0.10688</v>
       </c>
       <c r="J37" t="n">
-        <v>0.4990999999999999</v>
+        <v>0.5312599999999998</v>
       </c>
     </row>
     <row r="38">
@@ -1930,22 +1930,22 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.2171</v>
+        <v>0.13694</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2256</v>
+        <v>0.13936</v>
       </c>
       <c r="G38" t="n">
-        <v>0.4359</v>
+        <v>0.39246</v>
       </c>
       <c r="H38" t="n">
-        <v>0.7282</v>
+        <v>0.70244</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2838000000000001</v>
+        <v>0.2640799999999999</v>
       </c>
       <c r="J38" t="n">
-        <v>0.4136</v>
+        <v>0.5188600000000001</v>
       </c>
     </row>
     <row r="39">
@@ -1970,22 +1970,22 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.5009</v>
+        <v>0.4010199999999999</v>
       </c>
       <c r="F39" t="n">
-        <v>0.5231</v>
+        <v>0.42766</v>
       </c>
       <c r="G39" t="n">
-        <v>0.6513</v>
+        <v>0.5763999999999999</v>
       </c>
       <c r="H39" t="n">
-        <v>0.8769</v>
+        <v>0.85436</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2838000000000001</v>
+        <v>0.2640799999999999</v>
       </c>
       <c r="J39" t="n">
-        <v>0.4136</v>
+        <v>0.5188600000000001</v>
       </c>
     </row>
     <row r="40">
@@ -2010,22 +2010,22 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.9145</v>
+        <v>0.91988</v>
       </c>
       <c r="F40" t="n">
-        <v>0.9333</v>
+        <v>0.93686</v>
       </c>
       <c r="G40" t="n">
-        <v>0.9077</v>
+        <v>0.9229800000000001</v>
       </c>
       <c r="H40" t="n">
-        <v>1</v>
+        <v>0.99796</v>
       </c>
       <c r="I40" t="n">
-        <v>0.2838000000000001</v>
+        <v>0.2640799999999999</v>
       </c>
       <c r="J40" t="n">
-        <v>0.4136</v>
+        <v>0.5188600000000001</v>
       </c>
     </row>
     <row r="41">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+          <t>{"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2050,22 +2050,22 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>0.1043</v>
+        <v>0.12266</v>
       </c>
       <c r="F41" t="n">
-        <v>0.1154</v>
+        <v>0.13026</v>
       </c>
       <c r="G41" t="n">
-        <v>0.3436</v>
+        <v>0.36066</v>
       </c>
       <c r="H41" t="n">
-        <v>0.6974</v>
+        <v>0.72624</v>
       </c>
       <c r="I41" t="n">
-        <v>0.1948</v>
+        <v>0.17786</v>
       </c>
       <c r="J41" t="n">
-        <v>0.6086</v>
+        <v>0.5961000000000001</v>
       </c>
     </row>
     <row r="42">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+          <t>{"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2090,22 +2090,22 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.2991</v>
+        <v>0.30052</v>
       </c>
       <c r="F42" t="n">
-        <v>0.3231</v>
+        <v>0.32104</v>
       </c>
       <c r="G42" t="n">
-        <v>0.4872</v>
+        <v>0.4995</v>
       </c>
       <c r="H42" t="n">
-        <v>0.8308</v>
+        <v>0.8194800000000001</v>
       </c>
       <c r="I42" t="n">
-        <v>0.1948</v>
+        <v>0.17786</v>
       </c>
       <c r="J42" t="n">
-        <v>0.6086</v>
+        <v>0.5961000000000001</v>
       </c>
     </row>
     <row r="43">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}</t>
+          <t>{"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2130,22 +2130,22 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.9077</v>
+        <v>0.8966200000000001</v>
       </c>
       <c r="F43" t="n">
-        <v>0.9256</v>
+        <v>0.9163</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9282</v>
+        <v>0.91478</v>
       </c>
       <c r="H43" t="n">
-        <v>0.9949</v>
+        <v>0.9927800000000001</v>
       </c>
       <c r="I43" t="n">
-        <v>0.1948</v>
+        <v>0.17786</v>
       </c>
       <c r="J43" t="n">
-        <v>0.6086</v>
+        <v>0.5961000000000001</v>
       </c>
     </row>
     <row r="44">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}}</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2170,22 +2170,22 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.4564</v>
+        <v>0.30772</v>
       </c>
       <c r="F44" t="n">
-        <v>0.4872</v>
+        <v>0.3299</v>
       </c>
       <c r="G44" t="n">
-        <v>0.6051</v>
+        <v>0.49478</v>
       </c>
       <c r="H44" t="n">
-        <v>0.8462</v>
+        <v>0.8108999999999998</v>
       </c>
       <c r="I44" t="n">
-        <v>-0.03759999999999997</v>
+        <v>0.08167999999999997</v>
       </c>
       <c r="J44" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5414600000000001</v>
       </c>
     </row>
     <row r="45">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}}</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2210,22 +2210,22 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.4188</v>
+        <v>0.3894</v>
       </c>
       <c r="F45" t="n">
-        <v>0.4513</v>
+        <v>0.41434</v>
       </c>
       <c r="G45" t="n">
-        <v>0.5282</v>
+        <v>0.5292199999999999</v>
       </c>
       <c r="H45" t="n">
-        <v>0.8974</v>
+        <v>0.86668</v>
       </c>
       <c r="I45" t="n">
-        <v>-0.03759999999999997</v>
+        <v>0.08167999999999997</v>
       </c>
       <c r="J45" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5414600000000001</v>
       </c>
     </row>
     <row r="46">
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.248147, "environmental": 0.24439, "comfort": 0.202824, "practicality": 0.304639}}</t>
+          <t>{"HVAC": {"energy_cost": 0.138244, "environmental": 0.127688, "comfort": 0.662899, "practicality": 0.071169}, "Appliance": {"energy_cost": 0.207971, "environmental": 0.043979, "comfort": 0.29187, "practicality": 0.45618}, "Shower": {"energy_cost": 0.250328, "environmental": 0.246522, "comfort": 0.196918, "practicality": 0.306231}}</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2250,22 +2250,22 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.9385</v>
+        <v>0.93086</v>
       </c>
       <c r="F46" t="n">
-        <v>0.9487</v>
+        <v>0.9424800000000001</v>
       </c>
       <c r="G46" t="n">
-        <v>0.9538</v>
+        <v>0.94148</v>
       </c>
       <c r="H46" t="n">
-        <v>0.9949</v>
+        <v>0.9927800000000001</v>
       </c>
       <c r="I46" t="n">
-        <v>-0.03759999999999997</v>
+        <v>0.08167999999999997</v>
       </c>
       <c r="J46" t="n">
-        <v>0.5197000000000001</v>
+        <v>0.5414600000000001</v>
       </c>
     </row>
     <row r="47">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+          <t>{"energy_cost": 0.268909, "environmental": 0.371359, "comfort": 0.160782, "practicality": 0.19895}</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2290,22 +2290,22 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.1487</v>
+        <v>0.1226</v>
       </c>
       <c r="F47" t="n">
-        <v>0.1564</v>
+        <v>0.12814</v>
       </c>
       <c r="G47" t="n">
-        <v>0.3795</v>
+        <v>0.35128</v>
       </c>
       <c r="H47" t="n">
-        <v>0.7128</v>
+        <v>0.71898</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1846</v>
+        <v>0.20118</v>
       </c>
       <c r="J47" t="n">
-        <v>0.5402</v>
+        <v>0.5413600000000001</v>
       </c>
     </row>
     <row r="48">
@@ -2321,7 +2321,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+          <t>{"energy_cost": 0.268909, "environmental": 0.371359, "comfort": 0.160782, "practicality": 0.19895}</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2330,22 +2330,22 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.3333</v>
+        <v>0.32378</v>
       </c>
       <c r="F48" t="n">
-        <v>0.3538</v>
+        <v>0.34258</v>
       </c>
       <c r="G48" t="n">
-        <v>0.5436</v>
+        <v>0.5323399999999999</v>
       </c>
       <c r="H48" t="n">
-        <v>0.8256</v>
+        <v>0.8112999999999999</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1846</v>
+        <v>0.20118</v>
       </c>
       <c r="J48" t="n">
-        <v>0.5402</v>
+        <v>0.5413600000000001</v>
       </c>
     </row>
     <row r="49">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.268298, "environmental": 0.370515, "comfort": 0.162689, "practicality": 0.198498}</t>
+          <t>{"energy_cost": 0.268909, "environmental": 0.371359, "comfort": 0.160782, "practicality": 0.19895}</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2370,22 +2370,22 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.8735000000000001</v>
+        <v>0.86514</v>
       </c>
       <c r="F49" t="n">
-        <v>0.8897</v>
+        <v>0.88088</v>
       </c>
       <c r="G49" t="n">
-        <v>0.9026</v>
+        <v>0.89116</v>
       </c>
       <c r="H49" t="n">
-        <v>0.9744</v>
+        <v>0.97434</v>
       </c>
       <c r="I49" t="n">
-        <v>0.1846</v>
+        <v>0.20118</v>
       </c>
       <c r="J49" t="n">
-        <v>0.5402</v>
+        <v>0.5413600000000001</v>
       </c>
     </row>
     <row r="50">
@@ -2410,22 +2410,22 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.2137</v>
+        <v>0.15854</v>
       </c>
       <c r="F50" t="n">
-        <v>0.2231</v>
+        <v>0.16028</v>
       </c>
       <c r="G50" t="n">
-        <v>0.4513</v>
+        <v>0.3917</v>
       </c>
       <c r="H50" t="n">
-        <v>0.7487</v>
+        <v>0.73558</v>
       </c>
       <c r="I50" t="n">
-        <v>0.1607</v>
+        <v>0.18438</v>
       </c>
       <c r="J50" t="n">
-        <v>0.4991</v>
+        <v>0.52906</v>
       </c>
     </row>
     <row r="51">
@@ -2450,22 +2450,22 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>0.3744</v>
+        <v>0.34292</v>
       </c>
       <c r="F51" t="n">
-        <v>0.3974</v>
+        <v>0.36922</v>
       </c>
       <c r="G51" t="n">
-        <v>0.5846</v>
+        <v>0.55178</v>
       </c>
       <c r="H51" t="n">
-        <v>0.8512999999999999</v>
+        <v>0.8348599999999999</v>
       </c>
       <c r="I51" t="n">
-        <v>0.1607</v>
+        <v>0.18438</v>
       </c>
       <c r="J51" t="n">
-        <v>0.4991</v>
+        <v>0.52906</v>
       </c>
     </row>
     <row r="52">
@@ -2490,22 +2490,22 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>0.8735000000000001</v>
+        <v>0.87198</v>
       </c>
       <c r="F52" t="n">
-        <v>0.8974</v>
+        <v>0.89374</v>
       </c>
       <c r="G52" t="n">
-        <v>0.8769</v>
+        <v>0.8860199999999999</v>
       </c>
       <c r="H52" t="n">
-        <v>0.9897</v>
+        <v>0.98458</v>
       </c>
       <c r="I52" t="n">
-        <v>0.1607</v>
+        <v>0.18438</v>
       </c>
       <c r="J52" t="n">
-        <v>0.4991</v>
+        <v>0.52906</v>
       </c>
     </row>
     <row r="53">
@@ -2530,22 +2530,22 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.1385</v>
+        <v>0.12874</v>
       </c>
       <c r="F53" t="n">
-        <v>0.1487</v>
+        <v>0.13012</v>
       </c>
       <c r="G53" t="n">
-        <v>0.3949</v>
+        <v>0.36458</v>
       </c>
       <c r="H53" t="n">
-        <v>0.6872</v>
+        <v>0.7127599999999999</v>
       </c>
       <c r="I53" t="n">
-        <v>0.2359</v>
+        <v>0.20184</v>
       </c>
       <c r="J53" t="n">
-        <v>0.4923</v>
+        <v>0.53184</v>
       </c>
     </row>
     <row r="54">
@@ -2570,22 +2570,22 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.3744</v>
+        <v>0.33058</v>
       </c>
       <c r="F54" t="n">
-        <v>0.3923</v>
+        <v>0.35078</v>
       </c>
       <c r="G54" t="n">
-        <v>0.5897</v>
+        <v>0.5425599999999999</v>
       </c>
       <c r="H54" t="n">
-        <v>0.8205</v>
+        <v>0.8102599999999999</v>
       </c>
       <c r="I54" t="n">
-        <v>0.2359</v>
+        <v>0.20184</v>
       </c>
       <c r="J54" t="n">
-        <v>0.4923</v>
+        <v>0.53184</v>
       </c>
     </row>
     <row r="55">
@@ -2610,22 +2610,22 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>0.8667</v>
+        <v>0.86242</v>
       </c>
       <c r="F55" t="n">
-        <v>0.8821</v>
+        <v>0.8783000000000001</v>
       </c>
       <c r="G55" t="n">
-        <v>0.8974</v>
+        <v>0.89116</v>
       </c>
       <c r="H55" t="n">
-        <v>0.9692</v>
+        <v>0.96716</v>
       </c>
       <c r="I55" t="n">
-        <v>0.2359</v>
+        <v>0.20184</v>
       </c>
       <c r="J55" t="n">
-        <v>0.4923</v>
+        <v>0.53184</v>
       </c>
     </row>
     <row r="56">
@@ -2641,7 +2641,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+          <t>{"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2650,22 +2650,22 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.1761</v>
+        <v>0.16868</v>
       </c>
       <c r="F56" t="n">
-        <v>0.1872</v>
+        <v>0.17556</v>
       </c>
       <c r="G56" t="n">
-        <v>0.3795</v>
+        <v>0.3708</v>
       </c>
       <c r="H56" t="n">
-        <v>0.7077</v>
+        <v>0.7230599999999999</v>
       </c>
       <c r="I56" t="n">
-        <v>0.1538</v>
+        <v>0.13662</v>
       </c>
       <c r="J56" t="n">
-        <v>0.5367999999999999</v>
+        <v>0.5440999999999999</v>
       </c>
     </row>
     <row r="57">
@@ -2681,7 +2681,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+          <t>{"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2690,22 +2690,22 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>0.3299</v>
+        <v>0.3053</v>
       </c>
       <c r="F57" t="n">
-        <v>0.3462</v>
+        <v>0.32052</v>
       </c>
       <c r="G57" t="n">
-        <v>0.5487</v>
+        <v>0.5251399999999999</v>
       </c>
       <c r="H57" t="n">
-        <v>0.8154</v>
+        <v>0.8061800000000001</v>
       </c>
       <c r="I57" t="n">
-        <v>0.1538</v>
+        <v>0.13662</v>
       </c>
       <c r="J57" t="n">
-        <v>0.5367999999999999</v>
+        <v>0.5440999999999999</v>
       </c>
     </row>
     <row r="58">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>{"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}</t>
+          <t>{"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2730,22 +2730,22 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.8667</v>
+        <v>0.8493999999999999</v>
       </c>
       <c r="F58" t="n">
-        <v>0.8846000000000001</v>
+        <v>0.8696200000000001</v>
       </c>
       <c r="G58" t="n">
-        <v>0.8923</v>
+        <v>0.8747400000000001</v>
       </c>
       <c r="H58" t="n">
-        <v>0.9744</v>
+        <v>0.9692000000000001</v>
       </c>
       <c r="I58" t="n">
-        <v>0.1538</v>
+        <v>0.13662</v>
       </c>
       <c r="J58" t="n">
-        <v>0.5367999999999999</v>
+        <v>0.5440999999999999</v>
       </c>
     </row>
     <row r="59">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}}</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2770,22 +2770,22 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.0974</v>
+        <v>0.08891999999999999</v>
       </c>
       <c r="F59" t="n">
-        <v>0.1026</v>
+        <v>0.08838</v>
       </c>
       <c r="G59" t="n">
-        <v>0.3795</v>
+        <v>0.34404</v>
       </c>
       <c r="H59" t="n">
-        <v>0.6974</v>
+        <v>0.70766</v>
       </c>
       <c r="I59" t="n">
-        <v>0.2975</v>
+        <v>0.26356</v>
       </c>
       <c r="J59" t="n">
-        <v>0.5094000000000001</v>
+        <v>0.5414</v>
       </c>
     </row>
     <row r="60">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}}</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2810,22 +2810,22 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.3949</v>
+        <v>0.35248</v>
       </c>
       <c r="F60" t="n">
-        <v>0.4205</v>
+        <v>0.3764</v>
       </c>
       <c r="G60" t="n">
-        <v>0.5949</v>
+        <v>0.5476800000000001</v>
       </c>
       <c r="H60" t="n">
-        <v>0.8667</v>
+        <v>0.8399999999999999</v>
       </c>
       <c r="I60" t="n">
-        <v>0.2975</v>
+        <v>0.26356</v>
       </c>
       <c r="J60" t="n">
-        <v>0.5094000000000001</v>
+        <v>0.5414</v>
       </c>
     </row>
     <row r="61">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.333611, "environmental": 0.313969, "comfort": 0.126582, "practicality": 0.225838}}</t>
+          <t>{"HVAC": {"energy_cost": 0.336451, "environmental": 0.32038, "comfort": 0.269486, "practicality": 0.073683}, "Appliance": {"energy_cost": 0.193182, "environmental": 0.465156, "comfort": 0.123615, "practicality": 0.218047}, "Shower": {"energy_cost": 0.336687, "environmental": 0.316863, "comfort": 0.118531, "practicality": 0.22792}}</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2850,22 +2850,502 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>0.9043</v>
+        <v>0.89388</v>
       </c>
       <c r="F61" t="n">
-        <v>0.9205</v>
+        <v>0.9091400000000001</v>
       </c>
       <c r="G61" t="n">
-        <v>0.9282</v>
+        <v>0.92506</v>
       </c>
       <c r="H61" t="n">
-        <v>0.9897</v>
+        <v>0.98254</v>
       </c>
       <c r="I61" t="n">
-        <v>0.2975</v>
+        <v>0.26356</v>
       </c>
       <c r="J61" t="n">
-        <v>0.5094000000000001</v>
+        <v>0.5414</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>merec hvac-type only</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138, "environmental": 0.128, "comfort": 0.663, "practicality": 0.071}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>0.24578</v>
+      </c>
+      <c r="F62" t="n">
+        <v>0.25402</v>
+      </c>
+      <c r="G62" t="n">
+        <v>0.45244</v>
+      </c>
+      <c r="H62" t="n">
+        <v>0.77782</v>
+      </c>
+      <c r="I62" t="n">
+        <v>0.18738</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0.49292</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>merec hvac-type only</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138, "environmental": 0.128, "comfort": 0.663, "practicality": 0.071}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>0.43316</v>
+      </c>
+      <c r="F63" t="n">
+        <v>0.46616</v>
+      </c>
+      <c r="G63" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="H63" t="n">
+        <v>0.8748800000000001</v>
+      </c>
+      <c r="I63" t="n">
+        <v>0.18738</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0.49292</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>merec hvac-type only</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.138, "environmental": 0.128, "comfort": 0.663, "practicality": 0.071}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>0.92608</v>
+      </c>
+      <c r="F64" t="n">
+        <v>0.9343</v>
+      </c>
+      <c r="G64" t="n">
+        <v>0.9363400000000001</v>
+      </c>
+      <c r="H64" t="n">
+        <v>0.9815200000000001</v>
+      </c>
+      <c r="I64" t="n">
+        <v>0.18738</v>
+      </c>
+      <c r="J64" t="n">
+        <v>0.49292</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>merec appliance-type only</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.208, "environmental": 0.044, "comfort": 0.292, "practicality": 0.456}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>0.25758</v>
+      </c>
+      <c r="F65" t="n">
+        <v>0.27326</v>
+      </c>
+      <c r="G65" t="n">
+        <v>0.44112</v>
+      </c>
+      <c r="H65" t="n">
+        <v>0.7820199999999999</v>
+      </c>
+      <c r="I65" t="n">
+        <v>0.09627999999999992</v>
+      </c>
+      <c r="J65" t="n">
+        <v>0.551</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>merec appliance-type only</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.208, "environmental": 0.044, "comfort": 0.292, "practicality": 0.456}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>0.35386</v>
+      </c>
+      <c r="F66" t="n">
+        <v>0.3728399999999999</v>
+      </c>
+      <c r="G66" t="n">
+        <v>0.5353600000000001</v>
+      </c>
+      <c r="H66" t="n">
+        <v>0.81334</v>
+      </c>
+      <c r="I66" t="n">
+        <v>0.09627999999999992</v>
+      </c>
+      <c r="J66" t="n">
+        <v>0.551</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>merec appliance-type only</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.208, "environmental": 0.044, "comfort": 0.292, "practicality": 0.456}, "Shower": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}}</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>0.90486</v>
+      </c>
+      <c r="F67" t="n">
+        <v>0.9158199999999999</v>
+      </c>
+      <c r="G67" t="n">
+        <v>0.9117</v>
+      </c>
+      <c r="H67" t="n">
+        <v>0.9774200000000001</v>
+      </c>
+      <c r="I67" t="n">
+        <v>0.09627999999999992</v>
+      </c>
+      <c r="J67" t="n">
+        <v>0.551</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>merec shower-type only</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>0.09372</v>
+      </c>
+      <c r="F68" t="n">
+        <v>0.09409999999999999</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0.3369</v>
+      </c>
+      <c r="H68" t="n">
+        <v>0.6932</v>
+      </c>
+      <c r="I68" t="n">
+        <v>0.16508</v>
+      </c>
+      <c r="J68" t="n">
+        <v>0.6398799999999999</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>merec shower-type only</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>0.2588</v>
+      </c>
+      <c r="F69" t="n">
+        <v>0.28564</v>
+      </c>
+      <c r="G69" t="n">
+        <v>0.4871800000000001</v>
+      </c>
+      <c r="H69" t="n">
+        <v>0.80616</v>
+      </c>
+      <c r="I69" t="n">
+        <v>0.16508</v>
+      </c>
+      <c r="J69" t="n">
+        <v>0.6398799999999999</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>merec shower-type only</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Appliance": {"energy_cost": 0.3, "environmental": 0.35, "comfort": 0.2, "practicality": 0.15}, "Shower": {"energy_cost": 0.248, "environmental": 0.244, "comfort": 0.203, "practicality": 0.305}}</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>0.8986799999999999</v>
+      </c>
+      <c r="F70" t="n">
+        <v>0.9157999999999999</v>
+      </c>
+      <c r="G70" t="n">
+        <v>0.91578</v>
+      </c>
+      <c r="H70" t="n">
+        <v>0.9887</v>
+      </c>
+      <c r="I70" t="n">
+        <v>0.16508</v>
+      </c>
+      <c r="J70" t="n">
+        <v>0.6398799999999999</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>entropy per-type (tab)</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Direct_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>0.08892</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0.08840000000000001</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0.343</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0.7087</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0.26562</v>
+      </c>
+      <c r="J71" t="n">
+        <v>0.538</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>entropy per-type (tab)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Example-Guided_LLM_Scoring</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>0.35454</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0.37898</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0.54972</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0.8410399999999999</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0.26562</v>
+      </c>
+      <c r="J72" t="n">
+        <v>0.538</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>deepseek</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>entropy per-type (tab)</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>{"HVAC": {"energy_cost": 0.336336, "environmental": 0.32032, "comfort": 0.269269, "practicality": 0.074074}, "Appliance": {"energy_cost": 0.193, "environmental": 0.465, "comfort": 0.124, "practicality": 0.218}, "Shower": {"energy_cost": 0.333666, "environmental": 0.313686, "comfort": 0.126873, "practicality": 0.225774}}</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>LLM-Parameterized_Reference_Scoring</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>0.89254</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0.9080999999999999</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0.924</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0.98254</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0.26562</v>
+      </c>
+      <c r="J73" t="n">
+        <v>0.538</v>
       </c>
     </row>
   </sheetData>

</xml_diff>